<commit_message>
dati: griglia rigoristi, Fiorentina Goncalves P. > Mastantuono > Beto (designati ufficiali 13/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/griglia_rigoristi_serie_a_2026_27.xlsx
+++ b/dati/griglia_rigoristi_serie_a_2026_27.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Rigoristi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rigoristi" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,15 +534,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Goncalves P.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mastantuono</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Beto</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Goncalves P.</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -648,7 +652,6 @@
           <t>Cataldi</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -820,7 +823,6 @@
           <t>Simeone</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">

</xml_diff>